<commit_message>
Resolve control service-space conflicts and consolidate current engineering handoff
</commit_message>
<xml_diff>
--- a/reports/shareable_20261005/technical/TECHNICAL_REVIEW.xlsx
+++ b/reports/shareable_20261005/technical/TECHNICAL_REVIEW.xlsx
@@ -12,12 +12,14 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Claims" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Room scenarios" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Funding quotes" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release decisions" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Parts register" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pressure screening" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pressure assumptions" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fasteners" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Display dimensions" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current release gates" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Control module placement" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release decisions" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Parts register" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pressure screening" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pressure assumptions" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fasteners" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Display dimensions" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Read me'!$A$1:$B$6</definedName>
@@ -30,18 +32,22 @@
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'Room scenarios'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Funding quotes'!$A$1:$M$16</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="4">'Funding quotes'!$1:$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Release decisions'!$A$1:$J$13</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="5">'Release decisions'!$1:$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Parts register'!$A$1:$F$16</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="6">'Parts register'!$1:$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Pressure screening'!$A$1:$K$16</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="7">'Pressure screening'!$1:$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Pressure assumptions'!$A$1:$B$4</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="8">'Pressure assumptions'!$1:$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Fasteners'!$A$1:$D$9</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="9">'Fasteners'!$1:$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Display dimensions'!$A$1:$F$494</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="10">'Display dimensions'!$1:$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Current release gates'!$A$1:$J$14</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="5">'Current release gates'!$1:$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Control module placement'!$A$1:$H$19</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="6">'Control module placement'!$1:$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Release decisions'!$A$1:$J$13</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="7">'Release decisions'!$1:$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Parts register'!$A$1:$F$16</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="8">'Parts register'!$1:$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Pressure screening'!$A$1:$K$16</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="9">'Pressure screening'!$1:$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Pressure assumptions'!$A$1:$B$4</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="10">'Pressure assumptions'!$1:$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Fasteners'!$A$1:$D$9</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="11">'Fasteners'!$1:$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'Display dimensions'!$A$1:$F$494</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="12">'Display dimensions'!$1:$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -565,6 +571,685 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
+  <dimension ref="A1:K16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>total_m3h</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>per_filter_m3h</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>reducer_K</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>fan_Pa</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>plenum_Pa</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>inner_guard_Pa</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>outer_guard_Pa</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>installation_Pa</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>reducer_Pa</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>nonfilter_Pa</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>filter_allowance_Pa</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="38" customHeight="1">
+      <c r="A2" s="2" t="n">
+        <v>200</v>
+      </c>
+      <c r="B2" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D2" s="2" t="n">
+        <v>32.59998230680289</v>
+      </c>
+      <c r="E2" s="2" t="n">
+        <v>0.8677361498395474</v>
+      </c>
+      <c r="F2" s="2" t="n">
+        <v>2.208837426402051</v>
+      </c>
+      <c r="G2" s="2" t="n">
+        <v>2.208837426402051</v>
+      </c>
+      <c r="H2" s="2" t="n">
+        <v>0.5784907665596982</v>
+      </c>
+      <c r="I2" s="2" t="n">
+        <v>0.02592105276800554</v>
+      </c>
+      <c r="J2" s="2" t="n">
+        <v>5.889822821971354</v>
+      </c>
+      <c r="K2" s="2" t="n">
+        <v>26.71015948483153</v>
+      </c>
+    </row>
+    <row r="3" ht="38" customHeight="1">
+      <c r="A3" s="3" t="n">
+        <v>200</v>
+      </c>
+      <c r="B3" s="3" t="n">
+        <v>100</v>
+      </c>
+      <c r="C3" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D3" s="3" t="n">
+        <v>32.59998230680289</v>
+      </c>
+      <c r="E3" s="3" t="n">
+        <v>0.8677361498395474</v>
+      </c>
+      <c r="F3" s="3" t="n">
+        <v>2.208837426402051</v>
+      </c>
+      <c r="G3" s="3" t="n">
+        <v>2.208837426402051</v>
+      </c>
+      <c r="H3" s="3" t="n">
+        <v>0.5784907665596982</v>
+      </c>
+      <c r="I3" s="3" t="n">
+        <v>0.05184210553601108</v>
+      </c>
+      <c r="J3" s="3" t="n">
+        <v>5.915743874739359</v>
+      </c>
+      <c r="K3" s="3" t="n">
+        <v>26.68423843206353</v>
+      </c>
+    </row>
+    <row r="4" ht="38" customHeight="1">
+      <c r="A4" s="2" t="n">
+        <v>200</v>
+      </c>
+      <c r="B4" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="C4" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D4" s="2" t="n">
+        <v>32.59998230680289</v>
+      </c>
+      <c r="E4" s="2" t="n">
+        <v>0.8677361498395474</v>
+      </c>
+      <c r="F4" s="2" t="n">
+        <v>2.208837426402051</v>
+      </c>
+      <c r="G4" s="2" t="n">
+        <v>2.208837426402051</v>
+      </c>
+      <c r="H4" s="2" t="n">
+        <v>0.5784907665596982</v>
+      </c>
+      <c r="I4" s="2" t="n">
+        <v>0.1036842110720222</v>
+      </c>
+      <c r="J4" s="2" t="n">
+        <v>5.967585980275371</v>
+      </c>
+      <c r="K4" s="2" t="n">
+        <v>26.63239632652752</v>
+      </c>
+    </row>
+    <row r="5" ht="38" customHeight="1">
+      <c r="A5" s="3" t="n">
+        <v>250</v>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>125</v>
+      </c>
+      <c r="C5" s="3" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D5" s="3" t="n">
+        <v>30.09391027851171</v>
+      </c>
+      <c r="E5" s="3" t="n">
+        <v>1.355837734124293</v>
+      </c>
+      <c r="F5" s="3" t="n">
+        <v>3.451308478753206</v>
+      </c>
+      <c r="G5" s="3" t="n">
+        <v>3.451308478753206</v>
+      </c>
+      <c r="H5" s="3" t="n">
+        <v>0.9038918227495287</v>
+      </c>
+      <c r="I5" s="3" t="n">
+        <v>0.04050164495000866</v>
+      </c>
+      <c r="J5" s="3" t="n">
+        <v>9.202848159330243</v>
+      </c>
+      <c r="K5" s="3" t="n">
+        <v>20.89106211918147</v>
+      </c>
+    </row>
+    <row r="6" ht="38" customHeight="1">
+      <c r="A6" s="2" t="n">
+        <v>250</v>
+      </c>
+      <c r="B6" s="2" t="n">
+        <v>125</v>
+      </c>
+      <c r="C6" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" s="2" t="n">
+        <v>30.09391027851171</v>
+      </c>
+      <c r="E6" s="2" t="n">
+        <v>1.355837734124293</v>
+      </c>
+      <c r="F6" s="2" t="n">
+        <v>3.451308478753206</v>
+      </c>
+      <c r="G6" s="2" t="n">
+        <v>3.451308478753206</v>
+      </c>
+      <c r="H6" s="2" t="n">
+        <v>0.9038918227495287</v>
+      </c>
+      <c r="I6" s="2" t="n">
+        <v>0.08100328990001732</v>
+      </c>
+      <c r="J6" s="2" t="n">
+        <v>9.243349804280252</v>
+      </c>
+      <c r="K6" s="2" t="n">
+        <v>20.85056047423146</v>
+      </c>
+    </row>
+    <row r="7" ht="38" customHeight="1">
+      <c r="A7" s="3" t="n">
+        <v>250</v>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>125</v>
+      </c>
+      <c r="C7" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D7" s="3" t="n">
+        <v>30.09391027851171</v>
+      </c>
+      <c r="E7" s="3" t="n">
+        <v>1.355837734124293</v>
+      </c>
+      <c r="F7" s="3" t="n">
+        <v>3.451308478753206</v>
+      </c>
+      <c r="G7" s="3" t="n">
+        <v>3.451308478753206</v>
+      </c>
+      <c r="H7" s="3" t="n">
+        <v>0.9038918227495287</v>
+      </c>
+      <c r="I7" s="3" t="n">
+        <v>0.1620065798000346</v>
+      </c>
+      <c r="J7" s="3" t="n">
+        <v>9.324353094180269</v>
+      </c>
+      <c r="K7" s="3" t="n">
+        <v>20.76955718433144</v>
+      </c>
+    </row>
+    <row r="8" ht="38" customHeight="1">
+      <c r="A8" s="2" t="n">
+        <v>300</v>
+      </c>
+      <c r="B8" s="2" t="n">
+        <v>150</v>
+      </c>
+      <c r="C8" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D8" s="2" t="n">
+        <v>27.62649553528014</v>
+      </c>
+      <c r="E8" s="2" t="n">
+        <v>1.952406337138982</v>
+      </c>
+      <c r="F8" s="2" t="n">
+        <v>4.969884209404615</v>
+      </c>
+      <c r="G8" s="2" t="n">
+        <v>4.969884209404615</v>
+      </c>
+      <c r="H8" s="2" t="n">
+        <v>1.301604224759321</v>
+      </c>
+      <c r="I8" s="2" t="n">
+        <v>0.05832236872801246</v>
+      </c>
+      <c r="J8" s="2" t="n">
+        <v>13.25210134943555</v>
+      </c>
+      <c r="K8" s="2" t="n">
+        <v>14.3743941858446</v>
+      </c>
+    </row>
+    <row r="9" ht="38" customHeight="1">
+      <c r="A9" s="3" t="n">
+        <v>300</v>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>150</v>
+      </c>
+      <c r="C9" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D9" s="3" t="n">
+        <v>27.62649553528014</v>
+      </c>
+      <c r="E9" s="3" t="n">
+        <v>1.952406337138982</v>
+      </c>
+      <c r="F9" s="3" t="n">
+        <v>4.969884209404615</v>
+      </c>
+      <c r="G9" s="3" t="n">
+        <v>4.969884209404615</v>
+      </c>
+      <c r="H9" s="3" t="n">
+        <v>1.301604224759321</v>
+      </c>
+      <c r="I9" s="3" t="n">
+        <v>0.1166447374560249</v>
+      </c>
+      <c r="J9" s="3" t="n">
+        <v>13.31042371816356</v>
+      </c>
+      <c r="K9" s="3" t="n">
+        <v>14.31607181711659</v>
+      </c>
+    </row>
+    <row r="10" ht="38" customHeight="1">
+      <c r="A10" s="2" t="n">
+        <v>300</v>
+      </c>
+      <c r="B10" s="2" t="n">
+        <v>150</v>
+      </c>
+      <c r="C10" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D10" s="2" t="n">
+        <v>27.62649553528014</v>
+      </c>
+      <c r="E10" s="2" t="n">
+        <v>1.952406337138982</v>
+      </c>
+      <c r="F10" s="2" t="n">
+        <v>4.969884209404615</v>
+      </c>
+      <c r="G10" s="2" t="n">
+        <v>4.969884209404615</v>
+      </c>
+      <c r="H10" s="2" t="n">
+        <v>1.301604224759321</v>
+      </c>
+      <c r="I10" s="2" t="n">
+        <v>0.2332894749120498</v>
+      </c>
+      <c r="J10" s="2" t="n">
+        <v>13.42706845561958</v>
+      </c>
+      <c r="K10" s="2" t="n">
+        <v>14.19942707966056</v>
+      </c>
+    </row>
+    <row r="11" ht="38" customHeight="1">
+      <c r="A11" s="3" t="n">
+        <v>350</v>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>175</v>
+      </c>
+      <c r="C11" s="3" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D11" s="3" t="n">
+        <v>25.26773196530823</v>
+      </c>
+      <c r="E11" s="3" t="n">
+        <v>2.657441958883614</v>
+      </c>
+      <c r="F11" s="3" t="n">
+        <v>6.764564618356284</v>
+      </c>
+      <c r="G11" s="3" t="n">
+        <v>6.764564618356284</v>
+      </c>
+      <c r="H11" s="3" t="n">
+        <v>1.771627972589076</v>
+      </c>
+      <c r="I11" s="3" t="n">
+        <v>0.07938322410201697</v>
+      </c>
+      <c r="J11" s="3" t="n">
+        <v>18.03758239228728</v>
+      </c>
+      <c r="K11" s="3" t="n">
+        <v>7.230149573020956</v>
+      </c>
+    </row>
+    <row r="12" ht="38" customHeight="1">
+      <c r="A12" s="2" t="n">
+        <v>350</v>
+      </c>
+      <c r="B12" s="2" t="n">
+        <v>175</v>
+      </c>
+      <c r="C12" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D12" s="2" t="n">
+        <v>25.26773196530823</v>
+      </c>
+      <c r="E12" s="2" t="n">
+        <v>2.657441958883614</v>
+      </c>
+      <c r="F12" s="2" t="n">
+        <v>6.764564618356284</v>
+      </c>
+      <c r="G12" s="2" t="n">
+        <v>6.764564618356284</v>
+      </c>
+      <c r="H12" s="2" t="n">
+        <v>1.771627972589076</v>
+      </c>
+      <c r="I12" s="2" t="n">
+        <v>0.1587664482040339</v>
+      </c>
+      <c r="J12" s="2" t="n">
+        <v>18.11696561638929</v>
+      </c>
+      <c r="K12" s="2" t="n">
+        <v>7.150766348918939</v>
+      </c>
+    </row>
+    <row r="13" ht="38" customHeight="1">
+      <c r="A13" s="3" t="n">
+        <v>350</v>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>175</v>
+      </c>
+      <c r="C13" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D13" s="3" t="n">
+        <v>25.26773196530823</v>
+      </c>
+      <c r="E13" s="3" t="n">
+        <v>2.657441958883614</v>
+      </c>
+      <c r="F13" s="3" t="n">
+        <v>6.764564618356284</v>
+      </c>
+      <c r="G13" s="3" t="n">
+        <v>6.764564618356284</v>
+      </c>
+      <c r="H13" s="3" t="n">
+        <v>1.771627972589076</v>
+      </c>
+      <c r="I13" s="3" t="n">
+        <v>0.3175328964080679</v>
+      </c>
+      <c r="J13" s="3" t="n">
+        <v>18.27573206459333</v>
+      </c>
+      <c r="K13" s="3" t="n">
+        <v>6.991999900714905</v>
+      </c>
+    </row>
+    <row r="14" ht="38" customHeight="1">
+      <c r="A14" s="2" t="n">
+        <v>400</v>
+      </c>
+      <c r="B14" s="2" t="n">
+        <v>200</v>
+      </c>
+      <c r="C14" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D14" s="2" t="n">
+        <v>22.83386008460588</v>
+      </c>
+      <c r="E14" s="2" t="n">
+        <v>3.47094459935819</v>
+      </c>
+      <c r="F14" s="2" t="n">
+        <v>8.835349705608206</v>
+      </c>
+      <c r="G14" s="2" t="n">
+        <v>8.835349705608206</v>
+      </c>
+      <c r="H14" s="2" t="n">
+        <v>2.313963066238793</v>
+      </c>
+      <c r="I14" s="2" t="n">
+        <v>0.1036842110720222</v>
+      </c>
+      <c r="J14" s="2" t="n">
+        <v>23.55929128788542</v>
+      </c>
+      <c r="K14" s="2" t="n">
+        <v>-0.7254312032795305</v>
+      </c>
+    </row>
+    <row r="15" ht="38" customHeight="1">
+      <c r="A15" s="3" t="n">
+        <v>400</v>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>200</v>
+      </c>
+      <c r="C15" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D15" s="3" t="n">
+        <v>22.83386008460588</v>
+      </c>
+      <c r="E15" s="3" t="n">
+        <v>3.47094459935819</v>
+      </c>
+      <c r="F15" s="3" t="n">
+        <v>8.835349705608206</v>
+      </c>
+      <c r="G15" s="3" t="n">
+        <v>8.835349705608206</v>
+      </c>
+      <c r="H15" s="3" t="n">
+        <v>2.313963066238793</v>
+      </c>
+      <c r="I15" s="3" t="n">
+        <v>0.2073684221440443</v>
+      </c>
+      <c r="J15" s="3" t="n">
+        <v>23.66297549895744</v>
+      </c>
+      <c r="K15" s="3" t="n">
+        <v>-0.829115414351552</v>
+      </c>
+    </row>
+    <row r="16" ht="38" customHeight="1">
+      <c r="A16" s="2" t="n">
+        <v>400</v>
+      </c>
+      <c r="B16" s="2" t="n">
+        <v>200</v>
+      </c>
+      <c r="C16" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D16" s="2" t="n">
+        <v>22.83386008460588</v>
+      </c>
+      <c r="E16" s="2" t="n">
+        <v>3.47094459935819</v>
+      </c>
+      <c r="F16" s="2" t="n">
+        <v>8.835349705608206</v>
+      </c>
+      <c r="G16" s="2" t="n">
+        <v>8.835349705608206</v>
+      </c>
+      <c r="H16" s="2" t="n">
+        <v>2.313963066238793</v>
+      </c>
+      <c r="I16" s="2" t="n">
+        <v>0.4147368442880886</v>
+      </c>
+      <c r="J16" s="2" t="n">
+        <v>23.87034392110148</v>
+      </c>
+      <c r="K16" s="2" t="n">
+        <v>-1.036483836495599</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:K16"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:B4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="55" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Field</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="36" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>CONDITIONAL SCREEN - NOT ACTUAL FLOW</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="113" customHeight="1">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Assumptions</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>2800 rpm OEM numeric curve; equal sharing among four fans and two parallel filters; density1.2; guard K1.5 each; plenum K1.5 and installation K1 on fan-aperture velocity. Reducer K0.5/1/2. Loss coefficients unverified; reducer/plenum may overlap. Static/installed compatibility unresolved. No loaded filter curve.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="38" customHeight="1">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Filter data</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>No measured clean or loaded curve; allowance is not actual loss</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:B4"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:D9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -779,7 +1464,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -14742,6 +15427,1438 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
+  <dimension ref="A1:J14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="23.4" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="24.05" customWidth="1" min="4" max="4"/>
+    <col width="55" customWidth="1" min="5" max="5"/>
+    <col width="42.9" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="20.15" customWidth="1" min="9" max="9"/>
+    <col width="17.55" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Responsible_role_not_assigned_person</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>State</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Decision</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Required_work</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Closure_evidence</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Reviewer_name</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Disposition</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Evidence_file</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="53" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>M01</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Mechanical</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>OPEN INTERNAL</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Guard strength and reach</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Select material and justified load/probe criteria; assess perforations, welds, side seams and attachments; verify unpowered sample.</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Annotated calculation/drawing plus signed inspection result</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr"/>
+      <c r="H2" s="2" t="inlineStr"/>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr"/>
+    </row>
+    <row r="3" ht="53" customHeight="1">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>M02</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Mechanical</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>OPEN INTERNAL</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>Cabinet joints and stability</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>Check plywood/cleat grade, bolt bearing, edge distances, wood screw withdrawal, feet, whole mass/CG and cable pull; no lifting by lid.</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>Approved structural details and stability test record</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr"/>
+      <c r="H3" s="3" t="inlineStr"/>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="J3" s="3" t="inlineStr"/>
+    </row>
+    <row r="4" ht="53" customHeight="1">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>M03</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Mechanical</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>MIXED INPUT</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Filter seal and service</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Confirm exact filter frame/tolerance, gasket force/compression, flatness and feedthrough seals; verify safe supported removal.</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Revised stops/retainers and fit/leak evidence</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr"/>
+      <c r="H4" s="2" t="inlineStr"/>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr"/>
+    </row>
+    <row r="5" ht="53" customHeight="1">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>M04</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Mechanical and electrical</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>WAITING OEM</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>Fan harness and protected entry</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>ARCTIC and Noctua connector/cable dimensions pending; Noctua220175. Complete insert, clamp, bend and retention design when received.</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>OEM evidence and updated integrated CAD/drawing</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr"/>
+      <c r="H5" s="3" t="inlineStr"/>
+      <c r="I5" s="3" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="J5" s="3" t="inlineStr"/>
+    </row>
+    <row r="6" ht="53" customHeight="1">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>E01</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Electrical and mechanical</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>OPEN INTERNAL</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Hazard and protective function</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Determine applicable requirements; reconcile fixed guards, isolated servicing and present restart requirements before choosing circuitry.</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>Signed functional allocation and explicit requirement disposition</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr"/>
+      <c r="H6" s="2" t="inlineStr"/>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr"/>
+    </row>
+    <row r="7" ht="53" customHeight="1">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>E02</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>Electrical</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>OPEN INTERNAL</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>Rated circuit and enclosure</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>Select DC switching/protection/isolation, wire ratings, verified connectors and enclosure; check startup and auxiliary loads. No terminal guesses.</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>Circuit, cable schedule, ratings and physical layout</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr"/>
+      <c r="H7" s="3" t="inlineStr"/>
+      <c r="I7" s="3" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="J7" s="3" t="inlineStr"/>
+    </row>
+    <row r="8" ht="53" customHeight="1">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>E03</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Electrical</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>SITE AND PHYSICAL</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Commissioning</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Verify site supply and OEM adapter suitability; test isolation, stop/restart, supply recovery, abnormal/thermal behaviour under approved procedures.</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>Signed commissioning record before performance tests</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr"/>
+      <c r="H8" s="2" t="inlineStr"/>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr"/>
+    </row>
+    <row r="9" ht="53" customHeight="1">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>P01</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>Mechanical and test lead</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>PHYSICAL DATA</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>Filter duty</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>Obtain exact clean/loaded curve or safe measured pressure/flow points; include all installed losses.</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>Accepted operating point with margin and replacement rule</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr"/>
+      <c r="H9" s="3" t="inlineStr"/>
+      <c r="I9" s="3" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="J9" s="3" t="inlineStr"/>
+    </row>
+    <row r="10" ht="53" customHeight="1">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>T01</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Test lead and project lead</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>TEAM DECISION</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Acceptance targets and room</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>Agree indoor premises, measured flow/noise targets, room volume, instrument methods and PM test plan before trials.</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>Approved test plan and thresholds</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr"/>
+      <c r="H10" s="2" t="inlineStr"/>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr"/>
+    </row>
+    <row r="11" ht="53" customHeight="1">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>T02</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Test lead</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>AFTER RELEASE</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>Measured prototype results</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>Measure airflow, filter losses, bypass, noise, power and room PM with background/control observations.</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>Raw logs, calibration references and reviewed results</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr"/>
+      <c r="H11" s="3" t="inlineStr"/>
+      <c r="I11" s="3" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="J11" s="3" t="inlineStr"/>
+    </row>
+    <row r="12" ht="53" customHeight="1">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>C01</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Project lead and engineers</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>AFTER REVIEW</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Procurement and change control</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Confirm exact SKUs, quantities, real quotes, lead times and service scopes; authorize only released lines.</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>Approved BOM and revision-specific purchase/build authorization</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr"/>
+      <c r="H12" s="2" t="inlineStr"/>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr"/>
+    </row>
+    <row r="13" ht="53" customHeight="1">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>O01</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Separate future project</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>OUT OF INDOOR SCOPE</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>Public outdoor tower</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>Heat/rain/corrosion/tampering/anchoring and wind-dependent benefit require separate design and field validation.</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>Separate outdoor release; no bubble radius claimed</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr"/>
+      <c r="H13" s="3" t="inlineStr"/>
+      <c r="I13" s="3" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="J13" s="3" t="inlineStr"/>
+    </row>
+    <row r="14" ht="38" customHeight="1">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>D05</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Digital preparation</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>CLOSED DIGITAL ONLY</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>E04 assumed service-volume collisions</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>Actual dimensions/wiring remain E02 release scope</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>CURRENT_CONTROL_CHECKS.json; unchanged reservations mutually clear</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr"/>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>DIGITAL PASS / NO BUILD RELEASE</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>CURRENT_CONTROL_CHECKS.json</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:J14"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:H19"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="17.55" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="55" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Object</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Xmin</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Ymin</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Zmin</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Xmax</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Ymax</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Zmax</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="38" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>CB1_SIMPLIFIED_ENVELOPE</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>-150.0</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>-100.0</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>-70.08</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>150.0</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>100.0</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>50.0</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>ORIGINAL APPROXIMATE SHELL; not Hammond manufacturing geometry</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="38" customHeight="1">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>PL1_SIMPLIFIED_PANEL</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>-142.5</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>-92.5</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>-60.0</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>142.5</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>92.5</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>-58.3744</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>OEM285x185 outline; simplified rectangular proxy, contour/holes omitted except2 proposed4.5mm holes</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="38" customHeight="1">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>DIN1_ENVELOPE</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>-135.0</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>-17.5</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>-58.3744</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>-10.0</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>17.5</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>-50.8744</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>OEM35x7.5 profile envelope; proposed125mm cut, not full profile or approved attachment</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="38" customHeight="1">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>CTRL1_OPTA_LITE</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>-115.0</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>-44.4</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>-50.8744</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>-45.0</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>44.4</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>10.2256</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>OEM BODY DIMENSIONS / ASSUMED POSITION, ORIENTATION AND MOUNT; no connector geometry</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="38" customHeight="1">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>H1_NA_FH1</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>-15.0</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>-70.00000000000001</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>-53.3744</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>28.00000000000003</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>23.0</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>-40.8744</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>OEM BODY DIMENSIONS / ASSUMED POSITION, ORIENTATION AND MOUNT; no connector geometry</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="38" customHeight="1">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>SC1_NA_FC1</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>68.0</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>-65.0</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>-53.3744</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>116.0</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>-40.0</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>-32.3744</t>
+        </is>
+      </c>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>OEM BODY DIMENSIONS / ASSUMED POSITION, ORIENTATION AND MOUNT; no connector geometry</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="38" customHeight="1">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>CTRL1_WIRE_SPACE_ASSUMED</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>-125.0</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>-64.4</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>-50.8744</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>-35.0</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>64.4</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>10.2256</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>ASSUMED routing/service volume; actual connectors/clip release and bends unknown</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="38" customHeight="1">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>H1_CONNECTOR_SPACE_ASSUMED</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>-35.0</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>-80.00000000000001</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>-53.3744</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>48.00000000000003</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>33.00000000000001</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>-25.8744</t>
+        </is>
+      </c>
+      <c r="H9" s="3" t="inlineStr">
+        <is>
+          <t>ASSUMED routing/service volume; actual connectors/clip release and bends unknown</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="38" customHeight="1">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>SC1_CONNECTOR_SPACE_ASSUMED</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>58.0</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>-85.0</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>-53.3744</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>126.0</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>-20.0</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>-17.3744</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>ASSUMED routing/service volume; actual connectors/clip release and bends unknown</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="38" customHeight="1">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>START_FACE_PROXY</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>-29.5</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>40.5</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>50.0</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>-0.5</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>69.5</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>58.0</t>
+        </is>
+      </c>
+      <c r="H11" s="3" t="inlineStr">
+        <is>
+          <t>29mm head width from OEM; round face and 8mm projection ASSUMED</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="38" customHeight="1">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>START_REAR_ASSUMED</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>-35.0</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>35.0</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>-9.0</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>5.0</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>75.0</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>46.0</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>ASSUMED40x40x55 below inner lid; not assembled OEM dimensions</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="38" customHeight="1">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>START_WIRE_TAIL_ASSUMED</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>-35.0</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>35.0</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>-29.0</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>5.0</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>75.0</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>-9.0</t>
+        </is>
+      </c>
+      <c r="H13" s="3" t="inlineStr">
+        <is>
+          <t>ASSUMED20mm additional depth; not verified bend radius</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="38" customHeight="1">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>STOP_FACE_PROXY</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>30.5</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>40.5</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>50.0</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>59.5</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>69.5</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>58.0</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>29mm head width from OEM; round face and 8mm projection ASSUMED</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="38" customHeight="1">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>STOP_REAR_ASSUMED</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>25.0</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>35.0</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>-9.0</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>65.0</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>75.0</t>
+        </is>
+      </c>
+      <c r="G15" s="3" t="inlineStr">
+        <is>
+          <t>46.0</t>
+        </is>
+      </c>
+      <c r="H15" s="3" t="inlineStr">
+        <is>
+          <t>ASSUMED40x40x55 below inner lid; not assembled OEM dimensions</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="38" customHeight="1">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>STOP_WIRE_TAIL_ASSUMED</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>25.0</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>35.0</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>-29.0</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>65.0</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>75.0</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>-9.0</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>ASSUMED20mm additional depth; not verified bend radius</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="38" customHeight="1">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>RESET_FACE_PROXY</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>90.5</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>40.5</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>50.0</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>119.5</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>69.5</t>
+        </is>
+      </c>
+      <c r="G17" s="3" t="inlineStr">
+        <is>
+          <t>58.0</t>
+        </is>
+      </c>
+      <c r="H17" s="3" t="inlineStr">
+        <is>
+          <t>29mm head width from OEM; round face and 8mm projection ASSUMED</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="38" customHeight="1">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>RESET_REAR_ASSUMED</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>85.0</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>35.0</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>-9.0</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>125.0</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>75.0</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>46.0</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>ASSUMED40x40x55 below inner lid; not assembled OEM dimensions</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="38" customHeight="1">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>RESET_WIRE_TAIL_ASSUMED</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>85.0</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>35.0</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>-29.0</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>125.0</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>75.0</t>
+        </is>
+      </c>
+      <c r="G19" s="3" t="inlineStr">
+        <is>
+          <t>-9.0</t>
+        </is>
+      </c>
+      <c r="H19" s="3" t="inlineStr">
+        <is>
+          <t>ASSUMED20mm additional depth; not verified bend radius</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:H19"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:J13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -15296,7 +17413,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -15830,683 +17947,4 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="1"/>
-  </sheetPr>
-  <dimension ref="A1:K16"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="14" customWidth="1" min="10" max="10"/>
-    <col width="14" customWidth="1" min="11" max="11"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>total_m3h</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>per_filter_m3h</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>reducer_K</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>fan_Pa</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>plenum_Pa</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>inner_guard_Pa</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>outer_guard_Pa</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>installation_Pa</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>reducer_Pa</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>nonfilter_Pa</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>filter_allowance_Pa</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="38" customHeight="1">
-      <c r="A2" s="2" t="n">
-        <v>200</v>
-      </c>
-      <c r="B2" s="2" t="n">
-        <v>100</v>
-      </c>
-      <c r="C2" s="2" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="D2" s="2" t="n">
-        <v>32.59998230680289</v>
-      </c>
-      <c r="E2" s="2" t="n">
-        <v>0.8677361498395474</v>
-      </c>
-      <c r="F2" s="2" t="n">
-        <v>2.208837426402051</v>
-      </c>
-      <c r="G2" s="2" t="n">
-        <v>2.208837426402051</v>
-      </c>
-      <c r="H2" s="2" t="n">
-        <v>0.5784907665596982</v>
-      </c>
-      <c r="I2" s="2" t="n">
-        <v>0.02592105276800554</v>
-      </c>
-      <c r="J2" s="2" t="n">
-        <v>5.889822821971354</v>
-      </c>
-      <c r="K2" s="2" t="n">
-        <v>26.71015948483153</v>
-      </c>
-    </row>
-    <row r="3" ht="38" customHeight="1">
-      <c r="A3" s="3" t="n">
-        <v>200</v>
-      </c>
-      <c r="B3" s="3" t="n">
-        <v>100</v>
-      </c>
-      <c r="C3" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="D3" s="3" t="n">
-        <v>32.59998230680289</v>
-      </c>
-      <c r="E3" s="3" t="n">
-        <v>0.8677361498395474</v>
-      </c>
-      <c r="F3" s="3" t="n">
-        <v>2.208837426402051</v>
-      </c>
-      <c r="G3" s="3" t="n">
-        <v>2.208837426402051</v>
-      </c>
-      <c r="H3" s="3" t="n">
-        <v>0.5784907665596982</v>
-      </c>
-      <c r="I3" s="3" t="n">
-        <v>0.05184210553601108</v>
-      </c>
-      <c r="J3" s="3" t="n">
-        <v>5.915743874739359</v>
-      </c>
-      <c r="K3" s="3" t="n">
-        <v>26.68423843206353</v>
-      </c>
-    </row>
-    <row r="4" ht="38" customHeight="1">
-      <c r="A4" s="2" t="n">
-        <v>200</v>
-      </c>
-      <c r="B4" s="2" t="n">
-        <v>100</v>
-      </c>
-      <c r="C4" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="D4" s="2" t="n">
-        <v>32.59998230680289</v>
-      </c>
-      <c r="E4" s="2" t="n">
-        <v>0.8677361498395474</v>
-      </c>
-      <c r="F4" s="2" t="n">
-        <v>2.208837426402051</v>
-      </c>
-      <c r="G4" s="2" t="n">
-        <v>2.208837426402051</v>
-      </c>
-      <c r="H4" s="2" t="n">
-        <v>0.5784907665596982</v>
-      </c>
-      <c r="I4" s="2" t="n">
-        <v>0.1036842110720222</v>
-      </c>
-      <c r="J4" s="2" t="n">
-        <v>5.967585980275371</v>
-      </c>
-      <c r="K4" s="2" t="n">
-        <v>26.63239632652752</v>
-      </c>
-    </row>
-    <row r="5" ht="38" customHeight="1">
-      <c r="A5" s="3" t="n">
-        <v>250</v>
-      </c>
-      <c r="B5" s="3" t="n">
-        <v>125</v>
-      </c>
-      <c r="C5" s="3" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="D5" s="3" t="n">
-        <v>30.09391027851171</v>
-      </c>
-      <c r="E5" s="3" t="n">
-        <v>1.355837734124293</v>
-      </c>
-      <c r="F5" s="3" t="n">
-        <v>3.451308478753206</v>
-      </c>
-      <c r="G5" s="3" t="n">
-        <v>3.451308478753206</v>
-      </c>
-      <c r="H5" s="3" t="n">
-        <v>0.9038918227495287</v>
-      </c>
-      <c r="I5" s="3" t="n">
-        <v>0.04050164495000866</v>
-      </c>
-      <c r="J5" s="3" t="n">
-        <v>9.202848159330243</v>
-      </c>
-      <c r="K5" s="3" t="n">
-        <v>20.89106211918147</v>
-      </c>
-    </row>
-    <row r="6" ht="38" customHeight="1">
-      <c r="A6" s="2" t="n">
-        <v>250</v>
-      </c>
-      <c r="B6" s="2" t="n">
-        <v>125</v>
-      </c>
-      <c r="C6" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D6" s="2" t="n">
-        <v>30.09391027851171</v>
-      </c>
-      <c r="E6" s="2" t="n">
-        <v>1.355837734124293</v>
-      </c>
-      <c r="F6" s="2" t="n">
-        <v>3.451308478753206</v>
-      </c>
-      <c r="G6" s="2" t="n">
-        <v>3.451308478753206</v>
-      </c>
-      <c r="H6" s="2" t="n">
-        <v>0.9038918227495287</v>
-      </c>
-      <c r="I6" s="2" t="n">
-        <v>0.08100328990001732</v>
-      </c>
-      <c r="J6" s="2" t="n">
-        <v>9.243349804280252</v>
-      </c>
-      <c r="K6" s="2" t="n">
-        <v>20.85056047423146</v>
-      </c>
-    </row>
-    <row r="7" ht="38" customHeight="1">
-      <c r="A7" s="3" t="n">
-        <v>250</v>
-      </c>
-      <c r="B7" s="3" t="n">
-        <v>125</v>
-      </c>
-      <c r="C7" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="D7" s="3" t="n">
-        <v>30.09391027851171</v>
-      </c>
-      <c r="E7" s="3" t="n">
-        <v>1.355837734124293</v>
-      </c>
-      <c r="F7" s="3" t="n">
-        <v>3.451308478753206</v>
-      </c>
-      <c r="G7" s="3" t="n">
-        <v>3.451308478753206</v>
-      </c>
-      <c r="H7" s="3" t="n">
-        <v>0.9038918227495287</v>
-      </c>
-      <c r="I7" s="3" t="n">
-        <v>0.1620065798000346</v>
-      </c>
-      <c r="J7" s="3" t="n">
-        <v>9.324353094180269</v>
-      </c>
-      <c r="K7" s="3" t="n">
-        <v>20.76955718433144</v>
-      </c>
-    </row>
-    <row r="8" ht="38" customHeight="1">
-      <c r="A8" s="2" t="n">
-        <v>300</v>
-      </c>
-      <c r="B8" s="2" t="n">
-        <v>150</v>
-      </c>
-      <c r="C8" s="2" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="D8" s="2" t="n">
-        <v>27.62649553528014</v>
-      </c>
-      <c r="E8" s="2" t="n">
-        <v>1.952406337138982</v>
-      </c>
-      <c r="F8" s="2" t="n">
-        <v>4.969884209404615</v>
-      </c>
-      <c r="G8" s="2" t="n">
-        <v>4.969884209404615</v>
-      </c>
-      <c r="H8" s="2" t="n">
-        <v>1.301604224759321</v>
-      </c>
-      <c r="I8" s="2" t="n">
-        <v>0.05832236872801246</v>
-      </c>
-      <c r="J8" s="2" t="n">
-        <v>13.25210134943555</v>
-      </c>
-      <c r="K8" s="2" t="n">
-        <v>14.3743941858446</v>
-      </c>
-    </row>
-    <row r="9" ht="38" customHeight="1">
-      <c r="A9" s="3" t="n">
-        <v>300</v>
-      </c>
-      <c r="B9" s="3" t="n">
-        <v>150</v>
-      </c>
-      <c r="C9" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="D9" s="3" t="n">
-        <v>27.62649553528014</v>
-      </c>
-      <c r="E9" s="3" t="n">
-        <v>1.952406337138982</v>
-      </c>
-      <c r="F9" s="3" t="n">
-        <v>4.969884209404615</v>
-      </c>
-      <c r="G9" s="3" t="n">
-        <v>4.969884209404615</v>
-      </c>
-      <c r="H9" s="3" t="n">
-        <v>1.301604224759321</v>
-      </c>
-      <c r="I9" s="3" t="n">
-        <v>0.1166447374560249</v>
-      </c>
-      <c r="J9" s="3" t="n">
-        <v>13.31042371816356</v>
-      </c>
-      <c r="K9" s="3" t="n">
-        <v>14.31607181711659</v>
-      </c>
-    </row>
-    <row r="10" ht="38" customHeight="1">
-      <c r="A10" s="2" t="n">
-        <v>300</v>
-      </c>
-      <c r="B10" s="2" t="n">
-        <v>150</v>
-      </c>
-      <c r="C10" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="D10" s="2" t="n">
-        <v>27.62649553528014</v>
-      </c>
-      <c r="E10" s="2" t="n">
-        <v>1.952406337138982</v>
-      </c>
-      <c r="F10" s="2" t="n">
-        <v>4.969884209404615</v>
-      </c>
-      <c r="G10" s="2" t="n">
-        <v>4.969884209404615</v>
-      </c>
-      <c r="H10" s="2" t="n">
-        <v>1.301604224759321</v>
-      </c>
-      <c r="I10" s="2" t="n">
-        <v>0.2332894749120498</v>
-      </c>
-      <c r="J10" s="2" t="n">
-        <v>13.42706845561958</v>
-      </c>
-      <c r="K10" s="2" t="n">
-        <v>14.19942707966056</v>
-      </c>
-    </row>
-    <row r="11" ht="38" customHeight="1">
-      <c r="A11" s="3" t="n">
-        <v>350</v>
-      </c>
-      <c r="B11" s="3" t="n">
-        <v>175</v>
-      </c>
-      <c r="C11" s="3" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="D11" s="3" t="n">
-        <v>25.26773196530823</v>
-      </c>
-      <c r="E11" s="3" t="n">
-        <v>2.657441958883614</v>
-      </c>
-      <c r="F11" s="3" t="n">
-        <v>6.764564618356284</v>
-      </c>
-      <c r="G11" s="3" t="n">
-        <v>6.764564618356284</v>
-      </c>
-      <c r="H11" s="3" t="n">
-        <v>1.771627972589076</v>
-      </c>
-      <c r="I11" s="3" t="n">
-        <v>0.07938322410201697</v>
-      </c>
-      <c r="J11" s="3" t="n">
-        <v>18.03758239228728</v>
-      </c>
-      <c r="K11" s="3" t="n">
-        <v>7.230149573020956</v>
-      </c>
-    </row>
-    <row r="12" ht="38" customHeight="1">
-      <c r="A12" s="2" t="n">
-        <v>350</v>
-      </c>
-      <c r="B12" s="2" t="n">
-        <v>175</v>
-      </c>
-      <c r="C12" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D12" s="2" t="n">
-        <v>25.26773196530823</v>
-      </c>
-      <c r="E12" s="2" t="n">
-        <v>2.657441958883614</v>
-      </c>
-      <c r="F12" s="2" t="n">
-        <v>6.764564618356284</v>
-      </c>
-      <c r="G12" s="2" t="n">
-        <v>6.764564618356284</v>
-      </c>
-      <c r="H12" s="2" t="n">
-        <v>1.771627972589076</v>
-      </c>
-      <c r="I12" s="2" t="n">
-        <v>0.1587664482040339</v>
-      </c>
-      <c r="J12" s="2" t="n">
-        <v>18.11696561638929</v>
-      </c>
-      <c r="K12" s="2" t="n">
-        <v>7.150766348918939</v>
-      </c>
-    </row>
-    <row r="13" ht="38" customHeight="1">
-      <c r="A13" s="3" t="n">
-        <v>350</v>
-      </c>
-      <c r="B13" s="3" t="n">
-        <v>175</v>
-      </c>
-      <c r="C13" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="D13" s="3" t="n">
-        <v>25.26773196530823</v>
-      </c>
-      <c r="E13" s="3" t="n">
-        <v>2.657441958883614</v>
-      </c>
-      <c r="F13" s="3" t="n">
-        <v>6.764564618356284</v>
-      </c>
-      <c r="G13" s="3" t="n">
-        <v>6.764564618356284</v>
-      </c>
-      <c r="H13" s="3" t="n">
-        <v>1.771627972589076</v>
-      </c>
-      <c r="I13" s="3" t="n">
-        <v>0.3175328964080679</v>
-      </c>
-      <c r="J13" s="3" t="n">
-        <v>18.27573206459333</v>
-      </c>
-      <c r="K13" s="3" t="n">
-        <v>6.991999900714905</v>
-      </c>
-    </row>
-    <row r="14" ht="38" customHeight="1">
-      <c r="A14" s="2" t="n">
-        <v>400</v>
-      </c>
-      <c r="B14" s="2" t="n">
-        <v>200</v>
-      </c>
-      <c r="C14" s="2" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="D14" s="2" t="n">
-        <v>22.83386008460588</v>
-      </c>
-      <c r="E14" s="2" t="n">
-        <v>3.47094459935819</v>
-      </c>
-      <c r="F14" s="2" t="n">
-        <v>8.835349705608206</v>
-      </c>
-      <c r="G14" s="2" t="n">
-        <v>8.835349705608206</v>
-      </c>
-      <c r="H14" s="2" t="n">
-        <v>2.313963066238793</v>
-      </c>
-      <c r="I14" s="2" t="n">
-        <v>0.1036842110720222</v>
-      </c>
-      <c r="J14" s="2" t="n">
-        <v>23.55929128788542</v>
-      </c>
-      <c r="K14" s="2" t="n">
-        <v>-0.7254312032795305</v>
-      </c>
-    </row>
-    <row r="15" ht="38" customHeight="1">
-      <c r="A15" s="3" t="n">
-        <v>400</v>
-      </c>
-      <c r="B15" s="3" t="n">
-        <v>200</v>
-      </c>
-      <c r="C15" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="D15" s="3" t="n">
-        <v>22.83386008460588</v>
-      </c>
-      <c r="E15" s="3" t="n">
-        <v>3.47094459935819</v>
-      </c>
-      <c r="F15" s="3" t="n">
-        <v>8.835349705608206</v>
-      </c>
-      <c r="G15" s="3" t="n">
-        <v>8.835349705608206</v>
-      </c>
-      <c r="H15" s="3" t="n">
-        <v>2.313963066238793</v>
-      </c>
-      <c r="I15" s="3" t="n">
-        <v>0.2073684221440443</v>
-      </c>
-      <c r="J15" s="3" t="n">
-        <v>23.66297549895744</v>
-      </c>
-      <c r="K15" s="3" t="n">
-        <v>-0.829115414351552</v>
-      </c>
-    </row>
-    <row r="16" ht="38" customHeight="1">
-      <c r="A16" s="2" t="n">
-        <v>400</v>
-      </c>
-      <c r="B16" s="2" t="n">
-        <v>200</v>
-      </c>
-      <c r="C16" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="D16" s="2" t="n">
-        <v>22.83386008460588</v>
-      </c>
-      <c r="E16" s="2" t="n">
-        <v>3.47094459935819</v>
-      </c>
-      <c r="F16" s="2" t="n">
-        <v>8.835349705608206</v>
-      </c>
-      <c r="G16" s="2" t="n">
-        <v>8.835349705608206</v>
-      </c>
-      <c r="H16" s="2" t="n">
-        <v>2.313963066238793</v>
-      </c>
-      <c r="I16" s="2" t="n">
-        <v>0.4147368442880886</v>
-      </c>
-      <c r="J16" s="2" t="n">
-        <v>23.87034392110148</v>
-      </c>
-      <c r="K16" s="2" t="n">
-        <v>-1.036483836495599</v>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A1:K16"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="1"/>
-  </sheetPr>
-  <dimension ref="A1:B4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="55" customWidth="1" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Field</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Value</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="36" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>CONDITIONAL SCREEN - NOT ACTUAL FLOW</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="113" customHeight="1">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>Assumptions</t>
-        </is>
-      </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>2800 rpm OEM numeric curve; equal sharing among four fans and two parallel filters; density1.2; guard K1.5 each; plenum K1.5 and installation K1 on fan-aperture velocity. Reducer K0.5/1/2. Loss coefficients unverified; reducer/plenum may overlap. Static/installed compatibility unresolved. No loaded filter curve.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="38" customHeight="1">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>Filter data</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>No measured clean or loaded curve; allowance is not actual loss</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A1:B4"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
-</worksheet>
 </file>
</xml_diff>